<commit_message>
산출물(품질보안점검 v3-v4) 반영 + .gitignore(.vercel/.env.local)
- OPS-01: VM 내 일일 자동 백업 구축(예정→진행중) — cron 04:00 KST,
  sqlite3 .backup(WAL 포함), 14일 보관, 복원 검증. 오프서버 업로드(PAR)만 잔여
- SEC-09: 비밀번호 재설정 완료 처리(구현은 다음 커밋)
- vercel link가 추가한 .vercel/.env.local gitignore 항목

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/04_품질보안점검.xlsx
+++ b/docs/04_품질보안점검.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>이메일 발송 인프라는 구축됨 → 재설정 토큰 흐름 추가 예정</t>
+          <t>이메일 재설정 흐름 구현 — /auth/forgot(존재여부 비노출)→메일 링크 폼→/auth/reset(1시간·1회용 토큰). 회원 탈퇴(DELETE /auth/account, 비밀번호 재확인)도 함께</t>
         </is>
       </c>
     </row>
@@ -1045,12 +1045,12 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>진행중</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>단일 VM SQLite — cron으로 DB 파일 일 단위 복사 예정</t>
+          <t>VM 내 일일 자동 백업 구축(cron 04:00 KST, sqlite3 .backup — WAL 포함, gzip, 14일 보관, 복원 검증 완료). 남은 것: OCI Object Storage PAR 등록 시 오프서버 업로드(스크립트 준비됨)</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1393,6 +1393,40 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>OPS-01 갱신 — VM 내 일일 DB 백업 구축(예정→진행중), 오프서버 업로드만 잔여</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>SEC-09 완료 — 비밀번호 재설정 + 회원 탈퇴 구현</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:C2"/>
   <mergeCells count="1">

</xml_diff>